<commit_message>
update UI and add deletion scripts
</commit_message>
<xml_diff>
--- a/stock.xlsx
+++ b/stock.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github_place\Item-Level-Tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32260174-8599-40F7-BF90-2E4A80A9CE28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BAAA035-3BBD-46CE-B3ED-4273D086B774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="50">
   <si>
     <t>SKU</t>
   </si>
@@ -36,15 +36,6 @@
   </si>
   <si>
     <t>ID_PREFIX</t>
-  </si>
-  <si>
-    <t>Mũ đen</t>
-  </si>
-  <si>
-    <t>Mũ trắng</t>
-  </si>
-  <si>
-    <t>Túi 01</t>
   </si>
   <si>
     <t>Firestore Item Import Template</t>
@@ -122,13 +113,64 @@
     <t>The generated CSV includes ITEM_ID and QR_CONTENT for label generation.</t>
   </si>
   <si>
-    <t>MD</t>
+    <t>Lanyard</t>
   </si>
   <si>
-    <t>BAG</t>
+    <t>Áo thun thường</t>
   </si>
   <si>
-    <t>MT</t>
+    <t>Áo baby tee</t>
+  </si>
+  <si>
+    <t>Túi tote</t>
+  </si>
+  <si>
+    <t>Dây chuyền version 1</t>
+  </si>
+  <si>
+    <t>Dây chuyền version 2</t>
+  </si>
+  <si>
+    <t>Keyring 2 mảnh</t>
+  </si>
+  <si>
+    <t>Pin 1 - trường</t>
+  </si>
+  <si>
+    <t>Pin 2 - chương trình</t>
+  </si>
+  <si>
+    <t>Khăn bandana</t>
+  </si>
+  <si>
+    <t>TOTE</t>
+  </si>
+  <si>
+    <t>THUN</t>
+  </si>
+  <si>
+    <t>DC1</t>
+  </si>
+  <si>
+    <t>DC2</t>
+  </si>
+  <si>
+    <t>PIN1</t>
+  </si>
+  <si>
+    <t>PIN2</t>
+  </si>
+  <si>
+    <t>LAN</t>
+  </si>
+  <si>
+    <t>BABYT</t>
+  </si>
+  <si>
+    <t>KHAN</t>
+  </si>
+  <si>
+    <t>KEYR</t>
   </si>
 </sst>
 </file>
@@ -434,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2000"/>
+  <dimension ref="A1:E1996"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -463,96 +505,152 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>60</v>
+      </c>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3">
+        <v>200000</v>
+      </c>
+      <c r="D3">
+        <v>200</v>
+      </c>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4">
+        <v>180000</v>
+      </c>
+      <c r="D4">
+        <v>50</v>
+      </c>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5">
+        <v>100000</v>
+      </c>
+      <c r="D5">
+        <v>50</v>
+      </c>
+      <c r="E5" s="2"/>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>5</v>
+      <c r="C6">
+        <v>120000</v>
       </c>
-      <c r="C2" s="3">
-        <v>150000</v>
+      <c r="D6">
+        <v>100</v>
       </c>
-      <c r="D2" s="5">
-        <v>10</v>
+      <c r="E6" s="2"/>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="2" t="s">
+        <v>42</v>
       </c>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="2" t="s">
+      <c r="B7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7">
+        <v>30000</v>
+      </c>
+      <c r="D7">
+        <v>100</v>
+      </c>
+      <c r="E7" s="2"/>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>6</v>
+      <c r="C8">
+        <v>25000</v>
       </c>
-      <c r="C3" s="3">
-        <v>150000</v>
+      <c r="D8">
+        <v>50</v>
       </c>
-      <c r="D3" s="5">
-        <v>10</v>
+      <c r="E8" s="2"/>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="2" t="s">
+        <v>49</v>
       </c>
-      <c r="E3" s="2"/>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="2" t="s">
-        <v>34</v>
+      <c r="B9" s="2" t="s">
+        <v>36</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>7</v>
+      <c r="C9">
+        <v>40000</v>
       </c>
-      <c r="C4" s="3">
-        <v>220000</v>
+      <c r="D9">
+        <v>50</v>
       </c>
-      <c r="D4" s="5">
-        <v>10</v>
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="2" t="s">
+        <v>44</v>
       </c>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="2"/>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="2"/>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="2"/>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="5"/>
+      <c r="B10" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10">
+        <v>20000</v>
+      </c>
+      <c r="D10">
+        <v>50</v>
+      </c>
       <c r="E10" s="2"/>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="5"/>
+      <c r="A11" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11">
+        <v>25000</v>
+      </c>
+      <c r="D11">
+        <v>50</v>
+      </c>
       <c r="E11" s="2"/>
     </row>
     <row r="12" spans="1:5">
@@ -801,86 +899,74 @@
       <c r="E46" s="2"/>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="3"/>
-      <c r="D47" s="5"/>
-      <c r="E47" s="2"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="6"/>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="3"/>
-      <c r="D48" s="5"/>
-      <c r="E48" s="2"/>
-    </row>
-    <row r="49" spans="1:5">
-      <c r="A49" s="2"/>
-      <c r="B49" s="2"/>
-      <c r="C49" s="3"/>
-      <c r="D49" s="5"/>
-      <c r="E49" s="2"/>
-    </row>
-    <row r="50" spans="1:5">
-      <c r="A50" s="2"/>
-      <c r="B50" s="2"/>
-      <c r="C50" s="3"/>
-      <c r="D50" s="5"/>
-      <c r="E50" s="2"/>
-    </row>
-    <row r="51" spans="1:5">
+      <c r="C48" s="4"/>
+      <c r="D48" s="6"/>
+    </row>
+    <row r="49" spans="3:4">
+      <c r="C49" s="4"/>
+      <c r="D49" s="6"/>
+    </row>
+    <row r="50" spans="3:4">
+      <c r="C50" s="4"/>
+      <c r="D50" s="6"/>
+    </row>
+    <row r="51" spans="3:4">
       <c r="C51" s="4"/>
       <c r="D51" s="6"/>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="3:4">
       <c r="C52" s="4"/>
       <c r="D52" s="6"/>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="3:4">
       <c r="C53" s="4"/>
       <c r="D53" s="6"/>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="3:4">
       <c r="C54" s="4"/>
       <c r="D54" s="6"/>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="3:4">
       <c r="C55" s="4"/>
       <c r="D55" s="6"/>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="3:4">
       <c r="C56" s="4"/>
       <c r="D56" s="6"/>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="3:4">
       <c r="C57" s="4"/>
       <c r="D57" s="6"/>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="3:4">
       <c r="C58" s="4"/>
       <c r="D58" s="6"/>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="3:4">
       <c r="C59" s="4"/>
       <c r="D59" s="6"/>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="3:4">
       <c r="C60" s="4"/>
       <c r="D60" s="6"/>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="3:4">
       <c r="C61" s="4"/>
       <c r="D61" s="6"/>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="3:4">
       <c r="C62" s="4"/>
       <c r="D62" s="6"/>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="3:4">
       <c r="C63" s="4"/>
       <c r="D63" s="6"/>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="3:4">
       <c r="C64" s="4"/>
       <c r="D64" s="6"/>
     </row>
@@ -8611,22 +8697,6 @@
     <row r="1996" spans="3:4">
       <c r="C1996" s="4"/>
       <c r="D1996" s="6"/>
-    </row>
-    <row r="1997" spans="3:4">
-      <c r="C1997" s="4"/>
-      <c r="D1997" s="6"/>
-    </row>
-    <row r="1998" spans="3:4">
-      <c r="C1998" s="4"/>
-      <c r="D1998" s="6"/>
-    </row>
-    <row r="1999" spans="3:4">
-      <c r="C1999" s="4"/>
-      <c r="D1999" s="6"/>
-    </row>
-    <row r="2000" spans="3:4">
-      <c r="C2000" s="4"/>
-      <c r="D2000" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8645,7 +8715,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="21">
       <c r="A1" s="8" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -8653,10 +8723,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="7" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -8664,7 +8734,7 @@
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -8672,7 +8742,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -8680,7 +8750,7 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -8688,7 +8758,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -8696,20 +8766,20 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="9" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -8717,58 +8787,58 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" t="s">
         <v>19</v>
       </c>
-      <c r="B13" t="s">
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" t="s">
+      <c r="B15" t="s">
         <v>21</v>
       </c>
-      <c r="B14" t="s">
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
+      <c r="B16" t="s">
         <v>23</v>
       </c>
-      <c r="B15" t="s">
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" t="s">
+      <c r="B17" t="s">
         <v>25</v>
       </c>
-      <c r="B16" t="s">
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" t="s">
+      <c r="B18" t="s">
         <v>27</v>
       </c>
-      <c r="B17" t="s">
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" t="s">
+      <c r="B19" t="s">
         <v>29</v>
-      </c>
-      <c r="B18" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>